<commit_message>
Fix: Pass session to fetch_and_save_nodes to support authenticated subscription access
</commit_message>
<xml_diff>
--- a/套餐分析.xlsx
+++ b/套餐分析.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,153 +462,173 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>初级套餐</t>
+          <t>✦体验套餐✦TRIAL PACKAGE✦</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>32</v>
+        <v>14.82</v>
       </c>
       <c r="D2" t="n">
-        <v>250</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
+        <v>80</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>季付</t>
+          <t>月付</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>96</v>
+        <v>14.82</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>初级套餐</t>
+          <t>✦轻度使用✦LIGHT USE✦</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>27.5</v>
+        <v>22.8</v>
       </c>
       <c r="D3" t="n">
-        <v>250</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1000</v>
+        <v>110</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>年付</t>
+          <t>月付</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>330</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>中级套餐</t>
+          <t>✦轻度使用✦LIGHT USE✦</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="D4" t="n">
-        <v>500</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2000</v>
+        <v>110</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>月付</t>
+          <t>季付</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>中级套餐</t>
+          <t>✦轻度使用✦LIGHT USE✦</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>53.33</v>
+        <v>21.67</v>
       </c>
       <c r="D5" t="n">
-        <v>500</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2000</v>
+        <v>110</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>季付</t>
+          <t>半年付</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>160</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>中级套餐</t>
+          <t>✦轻度使用✦LIGHT USE✦</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>56.67</v>
+        <v>21.33</v>
       </c>
       <c r="D6" t="n">
-        <v>500</v>
-      </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2000</v>
+        <v>110</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -616,28 +636,30 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>680</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>高级套餐</t>
+          <t>✦中度使用✦MODERATE USE✦</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>120</v>
+        <v>43.8</v>
       </c>
       <c r="D7" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E7" t="n">
-        <v>5</v>
+        <v>260</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -646,32 +668,34 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>季付</t>
+          <t>月付</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>360</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>高级套餐</t>
+          <t>✦中度使用✦MODERATE USE✦</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100</v>
+        <v>42.67</v>
       </c>
       <c r="D8" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E8" t="n">
-        <v>5</v>
+        <v>260</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -680,32 +704,34 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>半年付</t>
+          <t>季付</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>600</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>高级套餐</t>
+          <t>✦中度使用✦MODERATE USE✦</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>80</v>
+        <v>41.67</v>
       </c>
       <c r="D9" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E9" t="n">
-        <v>5</v>
+        <v>260</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -714,11 +740,803 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>半年付</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>✦中度使用✦MODERATE USE✦</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>40.67</v>
+      </c>
+      <c r="D10" t="n">
+        <v>260</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>年付</t>
         </is>
       </c>
-      <c r="H9" t="n">
-        <v>960</v>
+      <c r="H10" t="n">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>420</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>59.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>56.67</v>
+      </c>
+      <c r="D12" t="n">
+        <v>420</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>53.33</v>
+      </c>
+      <c r="D13" t="n">
+        <v>420</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>半年付</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="n">
+        <v>420</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>✦深度使用✦DEEP USE✦</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>✦深度使用✦DEEP USE✦</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>92.67</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>✦深度使用✦DEEP USE✦</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>86</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>半年付</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>✦深度使用✦DEEP USE✦</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>83.25</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>225</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>222</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>216.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>半年付</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>207.33</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>✦轻度使用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="D23" t="n">
+        <v>130</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>✦中度使用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>40.67</v>
+      </c>
+      <c r="D24" t="n">
+        <v>338</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>✦重度使用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>50</v>
+      </c>
+      <c r="D25" t="n">
+        <v>500</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>✦深度使用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>83.25</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>✦小团队适用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>207.33</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2900</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>✦定制套餐✦CUSTOMIZED PACKAGE✦请联系客服再拍下✦</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>650</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>✦260G流量包(不限时)✦Unlimited time✦</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>260</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>一次性</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>✦550G流量包(不限时)✦Unlimited time✦</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>550</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>一次性</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>✦2200G流量包(不限时)✦Unlimited time✦</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>一次性</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>910</v>
       </c>
     </row>
   </sheetData>
@@ -732,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -785,22 +1603,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>高级套餐</t>
+          <t>✦深度使用✦年付特惠✦Annual discount✦</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>80</v>
+        <v>83.25</v>
       </c>
       <c r="D2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E2" t="n">
-        <v>5</v>
+        <v>1300</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -813,31 +1633,33 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>960</v>
+        <v>999</v>
       </c>
       <c r="I2" t="n">
-        <v>15</v>
+        <v>15.62</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>高级套餐</t>
+          <t>✦小团队适用✦年付特惠✦Annual discount✦</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>207.33</v>
       </c>
       <c r="D3" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
+        <v>2900</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -846,35 +1668,37 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>半年付</t>
+          <t>年付</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>600</v>
+        <v>2488</v>
       </c>
       <c r="I3" t="n">
-        <v>12</v>
+        <v>13.99</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>高级套餐</t>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>120</v>
+        <v>207.33</v>
       </c>
       <c r="D4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E4" t="n">
-        <v>5</v>
+        <v>2500</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -883,189 +1707,1067 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>季付</t>
+          <t>年付</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>360</v>
+        <v>2488</v>
       </c>
       <c r="I4" t="n">
-        <v>10</v>
+        <v>12.06</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>中级套餐</t>
+          <t>✦深度使用✦DEEP USE✦</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>53.33</v>
+        <v>83.25</v>
       </c>
       <c r="D5" t="n">
-        <v>500</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2000</v>
+        <v>1000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>季付</t>
+          <t>年付</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>160</v>
+        <v>999</v>
       </c>
       <c r="I5" t="n">
-        <v>9.380000000000001</v>
+        <v>12.01</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>初级套餐</t>
+          <t>✦深度使用✦DEEP USE✦</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27.5</v>
+        <v>86</v>
       </c>
       <c r="D6" t="n">
-        <v>250</v>
-      </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" t="n">
         <v>1000</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>年付</t>
+          <t>半年付</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>330</v>
+        <v>516</v>
       </c>
       <c r="I6" t="n">
-        <v>9.09</v>
+        <v>11.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>中级套餐</t>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>56.67</v>
+        <v>216.5</v>
       </c>
       <c r="D7" t="n">
-        <v>500</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2000</v>
+        <v>2500</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>年付</t>
+          <t>半年付</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>680</v>
+        <v>1299</v>
       </c>
       <c r="I7" t="n">
-        <v>8.82</v>
+        <v>11.55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>中级套餐</t>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>60</v>
+        <v>222</v>
       </c>
       <c r="D8" t="n">
-        <v>500</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2000</v>
+        <v>2500</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>月付</t>
+          <t>季付</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>60</v>
+        <v>666</v>
       </c>
       <c r="I8" t="n">
-        <v>8.33</v>
+        <v>11.26</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Viking Links</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>初级套餐</t>
+          <t>✦小团队适用✦SMALL TEAMS✦</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>32</v>
+        <v>225</v>
       </c>
       <c r="D9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>225</v>
+      </c>
+      <c r="I9" t="n">
+        <v>11.11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>✦深度使用✦DEEP USE✦</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>92.67</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>278</v>
+      </c>
+      <c r="I10" t="n">
+        <v>10.79</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>✦深度使用✦DEEP USE✦</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="I11" t="n">
+        <v>10.33</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>✦重度使用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="n">
+        <v>500</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>600</v>
+      </c>
+      <c r="I12" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="n">
+        <v>420</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>600</v>
+      </c>
+      <c r="I13" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>✦中度使用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>40.67</v>
+      </c>
+      <c r="D14" t="n">
+        <v>338</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>488</v>
+      </c>
+      <c r="I14" t="n">
+        <v>8.31</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>53.33</v>
+      </c>
+      <c r="D15" t="n">
+        <v>420</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>半年付</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>320</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7.88</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>56.67</v>
+      </c>
+      <c r="D16" t="n">
+        <v>420</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>170</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7.41</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>✦重度使用✦HEAVY USE✦</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="D17" t="n">
+        <v>420</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="I17" t="n">
+        <v>7.02</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>✦中度使用✦MODERATE USE✦</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>40.67</v>
+      </c>
+      <c r="D18" t="n">
+        <v>260</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>488</v>
+      </c>
+      <c r="I18" t="n">
+        <v>6.39</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>✦中度使用✦MODERATE USE✦</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="D19" t="n">
+        <v>260</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>半年付</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
         <v>250</v>
       </c>
-      <c r="E9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="I19" t="n">
+        <v>6.24</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>✦轻度使用✦年付特惠✦Annual discount✦</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="D20" t="n">
+        <v>130</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>256</v>
+      </c>
+      <c r="I20" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>✦中度使用✦MODERATE USE✦</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>42.67</v>
+      </c>
+      <c r="D21" t="n">
+        <v>260</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>128</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>✦中度使用✦MODERATE USE✦</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="D22" t="n">
+        <v>260</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="I22" t="n">
+        <v>5.94</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>✦体验套餐✦TRIAL PACKAGE✦</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="D23" t="n">
+        <v>80</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>✦轻度使用✦LIGHT USE✦</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="D24" t="n">
+        <v>110</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>年付</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>256</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5.16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>✦轻度使用✦LIGHT USE✦</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>21.67</v>
+      </c>
+      <c r="D25" t="n">
+        <v>110</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>半年付</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>130</v>
+      </c>
+      <c r="I25" t="n">
+        <v>5.08</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>✦轻度使用✦LIGHT USE✦</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>22</v>
+      </c>
+      <c r="D26" t="n">
+        <v>110</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>季付</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>66</v>
+      </c>
+      <c r="I26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>✦轻度使用✦LIGHT USE✦</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D27" t="n">
+        <v>110</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>月付</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="I27" t="n">
+        <v>4.82</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>✦定制套餐✦CUSTOMIZED PACKAGE✦请联系客服再拍下✦</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>650</v>
+      </c>
+      <c r="D28" t="n">
         <v>1000</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>季付</t>
         </is>
       </c>
-      <c r="H9" t="n">
-        <v>96</v>
-      </c>
-      <c r="I9" t="n">
-        <v>7.81</v>
+      <c r="H28" t="n">
+        <v>1950</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>✦260G流量包(不限时)✦Unlimited time✦</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>260</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>一次性</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>168</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>✦550G流量包(不限时)✦Unlimited time✦</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>550</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>一次性</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>268</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>UNi 独角兽机场</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>✦2200G流量包(不限时)✦Unlimited time✦</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>不限</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>一次性</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>910</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>